<commit_message>
Small changes in texts.
</commit_message>
<xml_diff>
--- a/LidarTotalBOM.xlsx
+++ b/LidarTotalBOM.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="87">
   <si>
     <t>No.</t>
   </si>
@@ -274,6 +274,9 @@
   </si>
   <si>
     <t>Chinese Avalanche photodiode NOT proved. Has IR filter modification</t>
+  </si>
+  <si>
+    <t>Original description: High-speed PTZ Motor DC12V Brushless ESC Drive</t>
   </si>
 </sst>
 </file>
@@ -309,7 +312,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -319,6 +322,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -336,7 +345,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
@@ -363,6 +372,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Гиперссылка" xfId="1" builtinId="8"/>
@@ -668,11 +678,11 @@
   <dimension ref="A1:G37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="5.88671875" customWidth="1"/>
+    <col min="2" max="2" width="8.33203125" customWidth="1"/>
     <col min="3" max="3" width="35.44140625" customWidth="1"/>
     <col min="4" max="4" width="12.44140625" style="8" customWidth="1"/>
     <col min="5" max="5" width="60.109375" style="4" customWidth="1"/>
-    <col min="6" max="6" width="49" style="6" customWidth="1"/>
+    <col min="6" max="6" width="40.77734375" style="6" customWidth="1"/>
     <col min="7" max="7" width="23.5546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -709,7 +719,7 @@
       <c r="E2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="12" t="s">
         <v>59</v>
       </c>
       <c r="G2" t="s">
@@ -730,7 +740,7 @@
       <c r="E3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="12" t="s">
         <v>79</v>
       </c>
     </row>
@@ -748,7 +758,7 @@
       <c r="E4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="12" t="s">
         <v>76</v>
       </c>
     </row>
@@ -858,7 +868,7 @@
       <c r="E11" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="F11" s="12" t="s">
         <v>60</v>
       </c>
     </row>
@@ -940,7 +950,7 @@
       <c r="E16" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="F16" s="5" t="s">
+      <c r="F16" s="12" t="s">
         <v>81</v>
       </c>
       <c r="G16" t="s">
@@ -960,8 +970,11 @@
       <c r="E17" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F17" s="5" t="s">
+      <c r="F17" s="12" t="s">
         <v>62</v>
+      </c>
+      <c r="G17" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.3">
@@ -977,7 +990,7 @@
       <c r="E18" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="F18" s="5" t="s">
+      <c r="F18" s="12" t="s">
         <v>83</v>
       </c>
       <c r="G18" t="s">
@@ -1012,7 +1025,7 @@
       <c r="E20" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F20" s="5" t="s">
+      <c r="F20" s="12" t="s">
         <v>63</v>
       </c>
     </row>
@@ -1029,7 +1042,7 @@
       <c r="E21" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="F21" s="5" t="s">
+      <c r="F21" s="12" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1046,7 +1059,7 @@
       <c r="E22" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="F22" s="5" t="s">
+      <c r="F22" s="12" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1085,7 +1098,7 @@
       <c r="E30" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="F30" s="5" t="s">
+      <c r="F30" s="12" t="s">
         <v>72</v>
       </c>
     </row>
@@ -1102,7 +1115,7 @@
       <c r="E31" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="F31" s="5" t="s">
+      <c r="F31" s="12" t="s">
         <v>66</v>
       </c>
     </row>
@@ -1147,7 +1160,7 @@
       <c r="E34" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="F34" s="5" t="s">
+      <c r="F34" s="12" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1175,8 +1188,8 @@
     <hyperlink ref="F16" r:id="rId12"/>
     <hyperlink ref="F17" r:id="rId13"/>
     <hyperlink ref="F33" r:id="rId14"/>
-    <hyperlink ref="F34" r:id="rId15" display="https://aliexpress.ru/item/32963619780.html"/>
-    <hyperlink ref="F31" r:id="rId16" display="https://aliexpress.ru/item/32735300921.html"/>
+    <hyperlink ref="F34" r:id="rId15"/>
+    <hyperlink ref="F31" r:id="rId16"/>
     <hyperlink ref="F18" r:id="rId17"/>
     <hyperlink ref="F10" r:id="rId18"/>
     <hyperlink ref="F11" r:id="rId19"/>

</xml_diff>